<commit_message>
Dicionário de dados, carts (1 por user_id) e (cart_items) (UNIQUE(cart_id, product_id) para não duplicar produto na mesma linha) .
</commit_message>
<xml_diff>
--- a/docs/Dicionario_Dados_ClubePlanner_SQLite.xlsx
+++ b/docs/Dicionario_Dados_ClubePlanner_SQLite.xlsx
@@ -173,7 +173,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -328,6 +328,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -582,8 +588,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:H95"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="14" customWidth="1" style="15" min="1" max="1"/>
     <col width="18" customWidth="1" style="15" min="2" max="2"/>
@@ -933,12 +939,16 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="16">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" t="inlineStr" s="36">
         <is>
           <t>PASSWORD_RESET_TOKENS</t>
         </is>
       </c>
-      <c r="B12" s="37" t="n"/>
+      <c r="B12" t="inlineStr" s="37">
+        <is>
+          <t/>
+        </is>
+      </c>
       <c r="C12" s="37" t="n"/>
       <c r="D12" s="37" t="n"/>
       <c r="E12" s="37" t="n"/>
@@ -2248,7 +2258,7 @@
     <row r="57">
       <c r="A57" s="44" t="inlineStr">
         <is>
-          <t>ORDERS</t>
+          <t>CARTS</t>
         </is>
       </c>
       <c r="B57" s="51" t="n"/>
@@ -2289,7 +2299,7 @@
       <c r="G58" s="46" t="n"/>
       <c r="H58" s="53" t="inlineStr">
         <is>
-          <t>Identificador único do pedido.</t>
+          <t>Identificador único do carrinho.</t>
         </is>
       </c>
     </row>
@@ -2307,184 +2317,178 @@
       </c>
       <c r="D59" s="42" t="inlineStr">
         <is>
+          <t>FK / UNIQUE</t>
+        </is>
+      </c>
+      <c r="E59" s="42" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F59" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G59" s="42" t="inlineStr">
+        <is>
+          <t>users.id</t>
+        </is>
+      </c>
+      <c r="H59" s="42" t="inlineStr">
+        <is>
+          <t>Dono do carrinho. Um carrinho por usuário logado (RF-07).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>datetime('now')</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Data de criação do carrinho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="44" t="inlineStr">
+        <is>
+          <t>CART_ITEMS</t>
+        </is>
+      </c>
+      <c r="B61" s="45" t="n"/>
+      <c r="C61" s="45" t="n"/>
+      <c r="D61" s="45" t="n"/>
+      <c r="E61" s="45" t="n"/>
+      <c r="F61" s="45" t="n"/>
+      <c r="G61" s="45" t="n"/>
+      <c r="H61" s="45" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="46" t="n"/>
+      <c r="B62" s="53" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C62" s="53" t="inlineStr">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="D62" s="46" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E62" s="53" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F62" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G62" s="46" t="n"/>
+      <c r="H62" s="53" t="inlineStr">
+        <is>
+          <t>Identificador único do item no carrinho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="42" t="n"/>
+      <c r="B63" s="56" t="inlineStr">
+        <is>
+          <t>cart_id</t>
+        </is>
+      </c>
+      <c r="C63" s="56" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D63" s="42" t="inlineStr">
+        <is>
           <t>FK</t>
         </is>
       </c>
-      <c r="E59" s="42" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F59" s="42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G59" s="42" t="inlineStr">
-        <is>
-          <t>users.id</t>
-        </is>
-      </c>
-      <c r="H59" s="42" t="inlineStr">
-        <is>
-          <t>Cliente que fez o pedido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="42" t="n"/>
-      <c r="B60" s="42" t="inlineStr">
-        <is>
-          <t>address_id</t>
-        </is>
-      </c>
-      <c r="C60" s="42" t="inlineStr">
+      <c r="E63" s="56" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F63" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G63" s="42" t="inlineStr">
+        <is>
+          <t>carts.id</t>
+        </is>
+      </c>
+      <c r="H63" s="56" t="inlineStr">
+        <is>
+          <t>Carrinho ao qual o item pertence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="42" t="n"/>
+      <c r="B64" s="56" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="C64" s="56" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="D60" s="42" t="inlineStr">
+      <c r="D64" s="42" t="inlineStr">
         <is>
           <t>FK</t>
         </is>
       </c>
-      <c r="E60" s="42" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F60" s="42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G60" s="42" t="inlineStr">
-        <is>
-          <t>addresses.id</t>
-        </is>
-      </c>
-      <c r="H60" s="42" t="inlineStr">
-        <is>
-          <t>Endereço de entrega selecionado no checkout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="42" t="n"/>
-      <c r="B61" s="42" t="inlineStr">
-        <is>
-          <t>coupon_id</t>
-        </is>
-      </c>
-      <c r="C61" s="42" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E61" s="42" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F61" s="42" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="G61" s="42" t="inlineStr">
-        <is>
-          <t>coupons.id</t>
-        </is>
-      </c>
-      <c r="H61" s="42" t="inlineStr">
-        <is>
-          <t>Cupom aplicado ao pedido, se houver (RF-08).</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="B62" s="15" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C62" s="15" t="inlineStr">
-        <is>
-          <t>TEXT CHECK (status IN ('pending','paid','shipped','delivered','canceled'))</t>
-        </is>
-      </c>
-      <c r="E62" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F62" s="15" t="inlineStr">
-        <is>
-          <t>'pending'</t>
-        </is>
-      </c>
-      <c r="H62" s="15" t="inlineStr">
-        <is>
-          <t>Status dinâmico do pedido (RF-10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>valor_total</t>
-        </is>
-      </c>
-      <c r="C63" s="15" t="inlineStr">
-        <is>
-          <t>REAL</t>
-        </is>
-      </c>
-      <c r="E63" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F63" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H63" s="15" t="inlineStr">
-        <is>
-          <t>Total do pedido recalculado no servidor (RN-01).</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="15" t="inlineStr">
-        <is>
-          <t>valor_frete</t>
-        </is>
-      </c>
-      <c r="C64" s="15" t="inlineStr">
-        <is>
-          <t>REAL</t>
-        </is>
-      </c>
-      <c r="E64" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F64" s="15" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-      <c r="H64" s="15" t="inlineStr">
-        <is>
-          <t>Valor do frete calculado por CEP (RF-07).</t>
+      <c r="E64" s="56" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F64" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G64" s="42" t="inlineStr">
+        <is>
+          <t>products.id</t>
+        </is>
+      </c>
+      <c r="H64" s="56" t="inlineStr">
+        <is>
+          <t>Produto adicionado ao carrinho.</t>
         </is>
       </c>
     </row>
@@ -2492,12 +2496,12 @@
       <c r="A65" s="55" t="n"/>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>valor_desconto</t>
+          <t>quantidade</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>INTEGER</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
@@ -2507,19 +2511,19 @@
       </c>
       <c r="F65" s="15" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H65" s="15" t="inlineStr">
         <is>
-          <t>Valor do desconto aplicado pelo cupom (RN-01: recalculado no servidor).</t>
+          <t>Quantidade do produto no carrinho.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>added_at</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
@@ -2539,14 +2543,14 @@
       </c>
       <c r="H66" s="15" t="inlineStr">
         <is>
-          <t>Data de criação do pedido.</t>
+          <t>Data em que o item foi adicionado. UNIQUE(cart_id, product_id) evita linha duplicada do mesmo produto.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="44" t="inlineStr">
         <is>
-          <t>ORDER_ITEMS</t>
+          <t>ORDERS</t>
         </is>
       </c>
       <c r="B67" s="45" t="n"/>
@@ -2587,7 +2591,7 @@
       <c r="G68" s="46" t="n"/>
       <c r="H68" s="53" t="inlineStr">
         <is>
-          <t>Identificador único do item do pedido.</t>
+          <t>Identificador único do pedido.</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2599,7 @@
       <c r="A69" s="42" t="n"/>
       <c r="B69" s="56" t="inlineStr">
         <is>
-          <t>order_id</t>
+          <t>user_id</t>
         </is>
       </c>
       <c r="C69" s="56" t="inlineStr">
@@ -2620,12 +2624,12 @@
       </c>
       <c r="G69" s="42" t="inlineStr">
         <is>
-          <t>orders.id</t>
+          <t>users.id</t>
         </is>
       </c>
       <c r="H69" s="56" t="inlineStr">
         <is>
-          <t>Pedido ao qual o item pertence.</t>
+          <t>Cliente que fez o pedido.</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2637,7 @@
       <c r="A70" s="42" t="n"/>
       <c r="B70" s="56" t="inlineStr">
         <is>
-          <t>product_id</t>
+          <t>address_id</t>
         </is>
       </c>
       <c r="C70" s="56" t="inlineStr">
@@ -2658,164 +2662,171 @@
       </c>
       <c r="G70" s="42" t="inlineStr">
         <is>
-          <t>products.id</t>
+          <t>addresses.id</t>
         </is>
       </c>
       <c r="H70" s="56" t="inlineStr">
         <is>
-          <t>Produto comprado.</t>
+          <t>Endereço de entrega selecionado no checkout.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="B71" s="15" t="inlineStr">
-        <is>
-          <t>quantidade</t>
-        </is>
-      </c>
-      <c r="C71" s="15" t="inlineStr">
+      <c r="A71" s="42" t="n"/>
+      <c r="B71" s="56" t="inlineStr">
+        <is>
+          <t>coupon_id</t>
+        </is>
+      </c>
+      <c r="C71" s="56" t="inlineStr">
         <is>
           <t>INTEGER</t>
         </is>
       </c>
-      <c r="E71" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F71" s="15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H71" s="15" t="inlineStr">
-        <is>
-          <t>Quantidade comprada do produto.</t>
+      <c r="D71" s="42" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E71" s="56" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F71" s="56" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="G71" s="42" t="inlineStr">
+        <is>
+          <t>coupons.id</t>
+        </is>
+      </c>
+      <c r="H71" s="56" t="inlineStr">
+        <is>
+          <t>Cupom aplicado ao pedido, se houver (RF-08).</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>preco_unitario</t>
+          <t>status</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
+          <t>TEXT CHECK (status IN ('pending','paid','shipped','delivered','canceled'))</t>
+        </is>
+      </c>
+      <c r="E72" s="15" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F72" s="15" t="inlineStr">
+        <is>
+          <t>'pending'</t>
+        </is>
+      </c>
+      <c r="H72" s="15" t="inlineStr">
+        <is>
+          <t>Status dinâmico do pedido (RF-10).</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="55" t="n"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>valor_total</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
           <t>REAL</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F72" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H72" s="15" t="inlineStr">
-        <is>
-          <t>Preço do produto no momento da compra (snapshot, não referencia products.preco).</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="44" t="inlineStr">
-        <is>
-          <t>PAYMENTS</t>
-        </is>
-      </c>
-      <c r="B73" s="45" t="n"/>
-      <c r="C73" s="45" t="n"/>
-      <c r="D73" s="45" t="n"/>
-      <c r="E73" s="45" t="n"/>
-      <c r="F73" s="45" t="n"/>
-      <c r="G73" s="45" t="n"/>
-      <c r="H73" s="45" t="n"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Total do pedido recalculado no servidor (RN-01).</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="46" t="n"/>
-      <c r="B74" s="53" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="C74" s="46" t="inlineStr">
-        <is>
-          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
-        </is>
-      </c>
-      <c r="D74" s="46" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E74" s="46" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F74" s="46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="46" t="n"/>
-      <c r="H74" s="46" t="inlineStr">
-        <is>
-          <t>Identificador único da transação.</t>
+      <c r="B74" s="15" t="inlineStr">
+        <is>
+          <t>valor_frete</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Valor do frete calculado por CEP (RF-07).</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="42" t="n"/>
-      <c r="B75" s="56" t="inlineStr">
-        <is>
-          <t>order_id</t>
-        </is>
-      </c>
-      <c r="C75" s="42" t="inlineStr">
-        <is>
-          <t>INTEGER</t>
-        </is>
-      </c>
-      <c r="D75" s="42" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E75" s="42" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F75" s="42" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="42" t="inlineStr">
-        <is>
-          <t>orders.id</t>
-        </is>
-      </c>
-      <c r="H75" s="42" t="inlineStr">
-        <is>
-          <t>Pedido relacionado ao pagamento.</t>
+      <c r="B75" s="15" t="inlineStr">
+        <is>
+          <t>valor_desconto</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Valor do desconto aplicado pelo cupom (RN-01: recalculado no servidor).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>metodo</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>TEXT CHECK (metodo IN ('pix','cartao','boleto'))</t>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
         </is>
       </c>
       <c r="E76" s="15" t="inlineStr">
@@ -2825,125 +2836,418 @@
       </c>
       <c r="F76" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>datetime('now')</t>
         </is>
       </c>
       <c r="H76" s="15" t="inlineStr">
         <is>
-          <t>Meio de pagamento usado no Checkout Transparente.</t>
+          <t>Data de criação do pedido.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="48" t="n"/>
-      <c r="B77" s="15" t="inlineStr">
-        <is>
-          <t>status_transacao</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t>TEXT CHECK (status_transacao IN ('approved','pending','authorized','in_process','in_mediation','rejected','cancelled','refunded','charged_back'))</t>
-        </is>
-      </c>
-      <c r="E77" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F77" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="inlineStr">
-        <is>
-          <t>Status retornado pela API do Mercado Pago. Domínio fechado com os 9 status reais (RN-02).</t>
-        </is>
-      </c>
+      <c r="A77" s="57" t="inlineStr">
+        <is>
+          <t>ORDER_ITEMS</t>
+        </is>
+      </c>
+      <c r="B77" s="51" t="n"/>
+      <c r="C77" s="51" t="n"/>
+      <c r="D77" s="45" t="n"/>
+      <c r="E77" s="51" t="n"/>
+      <c r="F77" s="51" t="n"/>
+      <c r="G77" s="45" t="n"/>
+      <c r="H77" s="51" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="15" t="inlineStr">
-        <is>
-          <t>transaction_id</t>
-        </is>
-      </c>
-      <c r="C78" s="15" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>UNIQUE</t>
-        </is>
-      </c>
-      <c r="E78" s="15" t="inlineStr">
-        <is>
-          <t>Sim</t>
-        </is>
-      </c>
-      <c r="F78" s="15" t="inlineStr">
-        <is>
-          <t>NULL</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="inlineStr">
-        <is>
-          <t>ID da transação no Mercado Pago (usado na validação do webhook). UNIQUE evita duplicidade em retries de webhook.</t>
+      <c r="A78" s="46" t="n"/>
+      <c r="B78" s="53" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C78" s="53" t="inlineStr">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="D78" s="53" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E78" s="53" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F78" s="53" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G78" s="46" t="n"/>
+      <c r="H78" s="53" t="inlineStr">
+        <is>
+          <t>Identificador único do item do pedido.</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="B79" s="15" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="C79" s="15" t="inlineStr">
-        <is>
-          <t>TEXT (ISO8601, default datetime('now'))</t>
-        </is>
-      </c>
-      <c r="E79" s="15" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="F79" s="15" t="inlineStr">
-        <is>
-          <t>datetime('now')</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="inlineStr">
-        <is>
-          <t>Última atualização do status (RN-02).</t>
+      <c r="A79" s="42" t="n"/>
+      <c r="B79" s="56" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="C79" s="56" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D79" s="42" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E79" s="56" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F79" s="56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G79" s="42" t="inlineStr">
+        <is>
+          <t>orders.id</t>
+        </is>
+      </c>
+      <c r="H79" s="56" t="inlineStr">
+        <is>
+          <t>Pedido ao qual o item pertence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="42" t="n"/>
+      <c r="B80" s="42" t="inlineStr">
+        <is>
+          <t>product_id</t>
+        </is>
+      </c>
+      <c r="C80" s="42" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D80" s="42" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E80" s="42" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F80" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G80" s="42" t="inlineStr">
+        <is>
+          <t>products.id</t>
+        </is>
+      </c>
+      <c r="H80" s="42" t="inlineStr">
+        <is>
+          <t>Produto comprado.</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="47" t="inlineStr">
-        <is>
-          <t>Legenda:</t>
+      <c r="A81" s="47" t="n"/>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>quantidade</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Quantidade comprada do produto.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="15" t="inlineStr">
         <is>
+          <t>preco_unitario</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Preço do produto no momento da compra (snapshot, não referencia products.preco).</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="44" t="inlineStr">
+        <is>
+          <t>PAYMENTS</t>
+        </is>
+      </c>
+      <c r="B83" s="51" t="n"/>
+      <c r="C83" s="45" t="n"/>
+      <c r="D83" s="45" t="n"/>
+      <c r="E83" s="45" t="n"/>
+      <c r="F83" s="45" t="n"/>
+      <c r="G83" s="45" t="n"/>
+      <c r="H83" s="45" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="46" t="n"/>
+      <c r="B84" s="46" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C84" s="46" t="inlineStr">
+        <is>
+          <t>INTEGER PRIMARY KEY AUTOINCREMENT</t>
+        </is>
+      </c>
+      <c r="D84" s="46" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="E84" s="46" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F84" s="46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G84" s="46" t="n"/>
+      <c r="H84" s="46" t="inlineStr">
+        <is>
+          <t>Identificador único da transação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="58" t="n"/>
+      <c r="B85" s="42" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="C85" s="42" t="inlineStr">
+        <is>
+          <t>INTEGER</t>
+        </is>
+      </c>
+      <c r="D85" s="42" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E85" s="42" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F85" s="42" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G85" s="42" t="inlineStr">
+        <is>
+          <t>orders.id</t>
+        </is>
+      </c>
+      <c r="H85" s="42" t="inlineStr">
+        <is>
+          <t>Pedido relacionado ao pagamento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>metodo</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>TEXT CHECK (metodo IN ('pix','cartao','boleto'))</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Meio de pagamento usado no Checkout Transparente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>status_transacao</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TEXT CHECK (status_transacao IN ('approved','pending','authorized','in_process','in_mediation','rejected','cancelled','refunded','charged_back'))</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Status retornado pela API do Mercado Pago. Domínio fechado com os 9 status reais (RN-02).</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>transaction_id</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TEXT</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>UNIQUE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>NULL</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>ID da transação no Mercado Pago (usado na validação do webhook). UNIQUE evita duplicidade em retries de webhook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TEXT (ISO8601, default datetime('now'))</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>datetime('now')</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Última atualização do status (RN-02).</t>
+        </is>
+      </c>
+    </row>
+    <row r="90"/>
+    <row r="91">
+      <c r="A91" s="47" t="inlineStr">
+        <is>
+          <t>Legenda:</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" t="inlineStr">
+        <is>
           <t>Amarelo = Chave primária (PK)</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="B83" s="15" t="inlineStr">
+    <row r="93">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Azul = Chave estrangeira (FK)</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="48" t="inlineStr">
+    <row r="94"/>
+    <row r="95">
+      <c r="A95" s="48" t="inlineStr">
         <is>
           <t>Nota: tipos, defaults e algumas regras (marcadas como "a definir") foram inferidos a partir da documentação do Notion (seção 03 - Modelagem do Banco de Dados, SRS e Arquitetura &amp; Segurança) e precisam de validação da equipe antes da migration.</t>
         </is>
@@ -2951,7 +3255,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A85:H85"/>
+    <mergeCell ref="A95:H95"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2965,8 +3269,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" style="15" min="1" max="1"/>
     <col width="14" customWidth="1" style="15" min="2" max="2"/>
@@ -3246,29 +3550,110 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>users</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>1 : N</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>password_reset_tokens</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>password_reset_tokens.user_id</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Um usuário pode solicitar várias recuperações de senha (RF-03).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>users</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1 : 1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>carts</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>carts.user_id</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Cada usuário logado tem no máximo um carrinho persistido (RF-07).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>carts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>cart_items</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cart_items.cart_id</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Um carrinho contém vários itens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>products</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1 : N</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>cart_items</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>cart_items.product_id</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Um produto pode estar em vários carrinhos.</t>
         </is>
       </c>
     </row>

</xml_diff>